<commit_message>
circuit breaker for api gateway and order service , invoked kafka for asynchronous mail services
</commit_message>
<xml_diff>
--- a/Backend/Microservices/SpringBoot-services/Shop Applications - URL Configuations.xlsx
+++ b/Backend/Microservices/SpringBoot-services/Shop Applications - URL Configuations.xlsx
@@ -8,15 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tech Stack\Projects\ShopApplication\Backend\Microservices\SpringBoot-services\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59F6299B-5B62-47D0-AD8C-F2E248675B46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DB94BD2-8A27-4647-B920-4C4579ED5D23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="URL Confiurations" sheetId="1" r:id="rId1"/>
-    <sheet name="KeyCloak" sheetId="2" r:id="rId2"/>
-    <sheet name="OAuth2 Configs" sheetId="3" r:id="rId3"/>
-    <sheet name="Token Details" sheetId="4" r:id="rId4"/>
+    <sheet name="kill server" sheetId="6" r:id="rId2"/>
+    <sheet name="mailtrap" sheetId="7" r:id="rId3"/>
+    <sheet name="Details" sheetId="5" r:id="rId4"/>
+    <sheet name="KeyCloak" sheetId="2" r:id="rId5"/>
+    <sheet name="OAuth2 Configs" sheetId="3" r:id="rId6"/>
+    <sheet name="Token Details" sheetId="4" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="89">
   <si>
     <t>Domain</t>
   </si>
@@ -47,9 +50,6 @@
     <t>Port</t>
   </si>
   <si>
-    <t>Path</t>
-  </si>
-  <si>
     <t>http://localhost</t>
   </si>
   <si>
@@ -104,9 +104,6 @@
     <t>Credentials</t>
   </si>
   <si>
-    <t>admin/admin</t>
-  </si>
-  <si>
     <t>root@keycloak/keycloak</t>
   </si>
   <si>
@@ -209,17 +206,133 @@
     <t>timestamp</t>
   </si>
   <si>
-    <t>shop-App-microservices-security-realm</t>
-  </si>
-  <si>
-    <t>shop-App-client-credentials</t>
+    <t>admin/adm!@#$%^&amp;*(_+)n</t>
+  </si>
+  <si>
+    <t>keycloak_db | MYSQL</t>
+  </si>
+  <si>
+    <t>ZooKeeper</t>
+  </si>
+  <si>
+    <t>To act as a cluster , as the kafka broker be run on cluster based</t>
+  </si>
+  <si>
+    <t>schema-registry</t>
+  </si>
+  <si>
+    <t>broker</t>
+  </si>
+  <si>
+    <t>kafka-ui</t>
+  </si>
+  <si>
+    <t>Provides an ui screen where we can see the messages and others</t>
+  </si>
+  <si>
+    <t>Services</t>
+  </si>
+  <si>
+    <t>Desc</t>
+  </si>
+  <si>
+    <t>depends on</t>
+  </si>
+  <si>
+    <t>broker , schema-registry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To avoid the conflicts between the producer and consumer's
+messages classes </t>
+  </si>
+  <si>
+    <t>docs.confluent.io</t>
+  </si>
+  <si>
+    <t>kafka.apache.org/</t>
+  </si>
+  <si>
+    <t>Document URL</t>
+  </si>
+  <si>
+    <t>mailtrap</t>
+  </si>
+  <si>
+    <t>mailtrap.io</t>
+  </si>
+  <si>
+    <t>Provides a free message email services</t>
+  </si>
+  <si>
+    <t>avro</t>
+  </si>
+  <si>
+    <t>provides the schema registry dependeny class creation</t>
+  </si>
+  <si>
+    <t>zookeeper</t>
+  </si>
+  <si>
+    <t>Path | Default Port</t>
+  </si>
+  <si>
+    <t>schema registry</t>
+  </si>
+  <si>
+    <t>shopApp-microservices-security-realm</t>
+  </si>
+  <si>
+    <t>Authentication flow</t>
+  </si>
+  <si>
+    <t>Service accounts roles</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <r>
+      <t>Client authentication</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cambria"/>
+        <family val="1"/>
+      </rPr>
+      <t> </t>
+    </r>
+  </si>
+  <si>
+    <t>notification-service</t>
+  </si>
+  <si>
+    <t>1)netstat -ano | findstr :1200
+2)taskkill /PID 15324 /F</t>
+  </si>
+  <si>
+    <t>1) Login with ar**********s**@gmail.com
+2) My Sandboxes</t>
+  </si>
+  <si>
+    <t>do not change the port to any other as no
+running error occurs</t>
+  </si>
+  <si>
+    <t>not used as avro is not 
+working sb 4.0.0+</t>
+  </si>
+  <si>
+    <t>a cluster needed for kafka 
+services</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -269,6 +382,53 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Cambria"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Cambria"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Cambria"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF151515"/>
+      <name val="Cambria"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Cambria"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Cambria"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -290,7 +450,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -418,12 +578,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyBorder="1"/>
@@ -435,9 +613,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -451,18 +627,86 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="23">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Cambria"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Cambria"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
     <dxf>
       <border outline="0">
         <top style="thin">
           <color theme="9"/>
         </top>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Cambria"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -493,6 +737,110 @@
         <left style="thin">
           <color indexed="64"/>
         </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
         <right/>
         <top style="thin">
           <color indexed="64"/>
@@ -689,26 +1037,42 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{586EC13A-0090-4C8A-B2F9-F8CBC5B0706D}" name="Table1" displayName="Table1" ref="C5:H16" headerRowDxfId="11" totalsRowDxfId="8" headerRowBorderDxfId="10" tableBorderDxfId="9">
-  <autoFilter ref="C5:H16" xr:uid="{586EC13A-0090-4C8A-B2F9-F8CBC5B0706D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{586EC13A-0090-4C8A-B2F9-F8CBC5B0706D}" name="Table1" displayName="Table1" ref="C5:H22" headerRowDxfId="22" totalsRowDxfId="19" headerRowBorderDxfId="21" tableBorderDxfId="20">
+  <autoFilter ref="C5:H22" xr:uid="{586EC13A-0090-4C8A-B2F9-F8CBC5B0706D}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C6:H22">
+    <sortCondition ref="D5:D22"/>
+  </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{94887A51-C6DC-4E40-973E-C815C42EA303}" name="Domain" totalsRowLabel="Total" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{95D35BD1-D864-41DA-BEFE-3298076F6F90}" name="Port" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{8F31824B-6FCA-4EFF-9661-2AC8FC65E7AD}" name="Path" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{36DA8933-3C90-44D9-996A-F581B5FD43DB}" name="App" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{F363270A-FFA1-4034-9378-478F866E2EBA}" name="Connected Services" totalsRowFunction="count" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{AA37D833-9C1F-4D47-A9A6-5487635F80DB}" name="Credentials" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{94887A51-C6DC-4E40-973E-C815C42EA303}" name="Domain" totalsRowLabel="Total" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{95D35BD1-D864-41DA-BEFE-3298076F6F90}" name="Port" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{8F31824B-6FCA-4EFF-9661-2AC8FC65E7AD}" name="Path | Default Port" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{36DA8933-3C90-44D9-996A-F581B5FD43DB}" name="App" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{F363270A-FFA1-4034-9378-478F866E2EBA}" name="Connected Services" totalsRowFunction="count" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{AA37D833-9C1F-4D47-A9A6-5487635F80DB}" name="Credentials" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{9200DD6E-7871-4054-AD38-2B1084E81186}" name="Table3" displayName="Table3" ref="C5:D8" totalsRowShown="0" headerRowDxfId="1" tableBorderDxfId="0">
-  <autoFilter ref="C5:D8" xr:uid="{9200DD6E-7871-4054-AD38-2B1084E81186}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2F482C16-A2DD-45DC-9DCF-D718694335E9}" name="Table2" displayName="Table2" ref="C5:F11" totalsRowShown="0" headerRowDxfId="12" headerRowBorderDxfId="11" tableBorderDxfId="10" totalsRowBorderDxfId="9">
+  <autoFilter ref="C5:F11" xr:uid="{2F482C16-A2DD-45DC-9DCF-D718694335E9}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{31E8A7A0-5E05-468D-AFB8-1E7C18628E95}" name="Services" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{77AA605D-8AD4-4141-A625-D1B2E877586E}" name="Document URL" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{9BB12546-D4BE-4AFB-8E5F-C19C09753E79}" name="Desc" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{D7C02557-C87C-4789-BE69-3BB9C5FAD87E}" name="depends on" dataDxfId="5"/>
+  </tableColumns>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{9200DD6E-7871-4054-AD38-2B1084E81186}" name="Table3" displayName="Table3" ref="C5:D11" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3" tableBorderDxfId="2">
+  <autoFilter ref="C5:D11" xr:uid="{9200DD6E-7871-4054-AD38-2B1084E81186}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{D040B9E5-D174-4300-941D-EE42421B92C1}" name="KeyCloak"/>
-    <tableColumn id="2" xr3:uid="{97E7EF84-4EBD-4899-B977-7A0AAA169098}" name="Config"/>
+    <tableColumn id="1" xr3:uid="{D040B9E5-D174-4300-941D-EE42421B92C1}" name="KeyCloak" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{97E7EF84-4EBD-4899-B977-7A0AAA169098}" name="Config" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -977,283 +1341,539 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C5:H16"/>
+  <dimension ref="C5:H22"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="3" max="3" width="24.33203125" customWidth="1"/>
-    <col min="4" max="4" width="32.1328125" customWidth="1"/>
-    <col min="5" max="5" width="20.46484375" customWidth="1"/>
-    <col min="6" max="6" width="19.53125" customWidth="1"/>
-    <col min="7" max="7" width="28.19921875" customWidth="1"/>
-    <col min="8" max="8" width="32.46484375" customWidth="1"/>
+    <col min="3" max="3" width="18.59765625" customWidth="1"/>
+    <col min="4" max="4" width="20.46484375" customWidth="1"/>
+    <col min="5" max="5" width="23.796875" customWidth="1"/>
+    <col min="6" max="6" width="26" customWidth="1"/>
+    <col min="7" max="7" width="21.1328125" customWidth="1"/>
+    <col min="8" max="8" width="23.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="5" spans="3:8" x14ac:dyDescent="0.45">
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="11" t="s">
         <v>0</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>2</v>
+        <v>76</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C6" s="7" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D6" s="1">
         <v>1000</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="9"/>
     </row>
     <row r="7" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C7" s="7" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" s="1">
-        <v>27017</v>
+        <v>1005</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="9"/>
     </row>
     <row r="8" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C8" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8" s="1">
+        <v>1010</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D8" s="1">
-        <v>1005</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>9</v>
-      </c>
       <c r="F8" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="9"/>
     </row>
     <row r="9" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C9" s="7" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D9" s="1">
-        <v>1010</v>
+        <v>1025</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G9" s="1"/>
       <c r="H9" s="9"/>
     </row>
     <row r="10" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C10" s="7" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" s="1">
-        <v>1025</v>
+        <v>1030</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G10" s="1"/>
       <c r="H10" s="9"/>
     </row>
     <row r="11" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C11" s="7" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D11" s="1">
-        <v>1030</v>
+        <v>1040</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="G11" s="1"/>
-      <c r="H11" s="9"/>
+      <c r="H11" s="21" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="12" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C12" s="7" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D12" s="1">
-        <v>2000</v>
+        <v>1050</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H12" s="9" t="s">
-        <v>8</v>
+        <v>55</v>
+      </c>
+      <c r="G12" s="1"/>
+      <c r="H12" s="21" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C13" s="7" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D13" s="1">
-        <v>2000</v>
+        <v>1060</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G13" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="H13" s="9" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="3:8" x14ac:dyDescent="0.45">
+      <c r="G13" s="1"/>
+      <c r="H13" s="9"/>
+    </row>
+    <row r="14" spans="3:8" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C14" s="7" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D14" s="1">
-        <v>2000</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>14</v>
-      </c>
+        <v>1070</v>
+      </c>
+      <c r="E14" s="1"/>
       <c r="F14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="3:8" x14ac:dyDescent="0.45">
-      <c r="C15" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="D15" s="1">
-        <v>1040</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G15" s="1"/>
-      <c r="H15" s="9" t="s">
-        <v>21</v>
+        <v>75</v>
+      </c>
+      <c r="G14" s="1"/>
+      <c r="H14" s="33" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="15" spans="3:8" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="C15" s="34" t="s">
+        <v>2</v>
+      </c>
+      <c r="D15" s="35">
+        <v>1100</v>
+      </c>
+      <c r="E15" s="35">
+        <v>8081</v>
+      </c>
+      <c r="F15" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="G15" s="35"/>
+      <c r="H15" s="36" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="16" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C16" s="10" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D16" s="4">
-        <v>1050</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>18</v>
+        <v>1100</v>
+      </c>
+      <c r="E16" s="4">
+        <v>8080</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>18</v>
+        <v>60</v>
       </c>
       <c r="G16" s="4"/>
-      <c r="H16" s="11" t="s">
-        <v>22</v>
+      <c r="H16" s="9"/>
+    </row>
+    <row r="17" spans="3:8" s="23" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="C17" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D17" s="4">
+        <v>1200</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G17" s="4"/>
+      <c r="H17" s="17"/>
+    </row>
+    <row r="18" spans="3:8" x14ac:dyDescent="0.45">
+      <c r="C18" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D18" s="4">
+        <v>2000</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H18" s="17"/>
+    </row>
+    <row r="19" spans="3:8" x14ac:dyDescent="0.45">
+      <c r="C19" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D19" s="4">
+        <v>2000</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="H19" s="17"/>
+    </row>
+    <row r="20" spans="3:8" x14ac:dyDescent="0.45">
+      <c r="C20" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D20" s="4">
+        <v>2000</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H20" s="17"/>
+    </row>
+    <row r="21" spans="3:8" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="C21" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D21" s="4">
+        <v>9092</v>
+      </c>
+      <c r="E21" s="4">
+        <v>9092</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G21" s="4"/>
+      <c r="H21" s="22" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="22" spans="3:8" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="C22" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D22" s="4">
+        <v>29092</v>
+      </c>
+      <c r="E22" s="4">
+        <v>29092</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G22" s="4"/>
+      <c r="H22" s="22" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C6" r:id="rId1" xr:uid="{DB41ACBE-58CC-414A-A716-E2CB637E3CC2}"/>
-    <hyperlink ref="C7" r:id="rId2" xr:uid="{F0275049-1D1F-483D-82E0-F0FA966B3196}"/>
-    <hyperlink ref="H16" r:id="rId3" xr:uid="{9F675A40-5D07-4703-AF92-D18C247A8318}"/>
+    <hyperlink ref="C13" r:id="rId2" xr:uid="{F0275049-1D1F-483D-82E0-F0FA966B3196}"/>
+    <hyperlink ref="H12" r:id="rId3" xr:uid="{9F675A40-5D07-4703-AF92-D18C247A8318}"/>
+    <hyperlink ref="H11" r:id="rId4" xr:uid="{C8599585-EEB0-428D-8AE1-1B227EFA7E20}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId5"/>
   <tableParts count="1">
-    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C1CC5C9-9106-4DFC-A494-E8B6BDA58048}">
+  <dimension ref="D4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="4" max="4" width="63.73046875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="4:4" ht="282.39999999999998" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="D4" s="31" t="s">
+        <v>84</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD77AA44-A0BA-459D-83FD-3D4E6A7D278D}">
+  <dimension ref="E7"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="5" max="5" width="57.265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="7" spans="5:5" ht="201.4" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E7" s="32" t="s">
+        <v>85</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB1B5230-650E-4675-B23E-2405B14CC1C7}">
+  <dimension ref="C5:F11"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="3" max="3" width="24.6640625" customWidth="1"/>
+    <col min="4" max="4" width="14.86328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.86328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="3:6" x14ac:dyDescent="0.45">
+      <c r="C5" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="3:6" x14ac:dyDescent="0.45">
+      <c r="C6" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" s="18"/>
+      <c r="E6" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="3:6" x14ac:dyDescent="0.45">
+      <c r="C7" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7" s="18"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="3:6" ht="57" x14ac:dyDescent="0.45">
+      <c r="C8" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="E8" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="F8" s="19" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="3:6" x14ac:dyDescent="0.45">
+      <c r="C9" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="3:6" x14ac:dyDescent="0.45">
+      <c r="C10" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="D10" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="3:6" x14ac:dyDescent="0.45">
+      <c r="C11" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="D11" s="18"/>
+      <c r="E11" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="F11" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0515376E-D51F-4813-B857-482397B74C80}">
-  <dimension ref="C5:D8"/>
+  <dimension ref="C5:D11"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="3" max="3" width="22.19921875" customWidth="1"/>
-    <col min="4" max="4" width="80.9296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="97.46484375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="5" spans="3:4" x14ac:dyDescent="0.45">
       <c r="C5" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D5" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="3:4" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="C6" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="7" spans="3:4" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="C7" s="26" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="6" spans="3:4" x14ac:dyDescent="0.45">
-      <c r="C6" s="2" t="s">
+      <c r="D7" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="7" spans="3:4" x14ac:dyDescent="0.45">
-      <c r="C7" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="8" spans="3:4" x14ac:dyDescent="0.45">
-      <c r="C8" t="s">
-        <v>31</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>32</v>
-      </c>
+    </row>
+    <row r="8" spans="3:4" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="C8" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="27" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="3:4" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="C9" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="D9" s="29" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="10" spans="3:4" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="C10" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="D10" s="26" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="3:4" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1266,7 +1886,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63AA1C63-49A1-44DA-ACE3-C78A922A9010}">
   <dimension ref="C7:D21"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1276,43 +1896,43 @@
   </cols>
   <sheetData>
     <row r="7" spans="3:4" x14ac:dyDescent="0.45">
-      <c r="C7" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>23</v>
+      <c r="C7" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.45">
       <c r="C8" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.45">
       <c r="C9" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.45">
       <c r="C10" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.45">
       <c r="C11" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.45">
@@ -1363,7 +1983,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5E80640-C9FF-4A02-96EF-87B640CCC02A}">
   <dimension ref="C6:C34"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1372,147 +1992,147 @@
   </cols>
   <sheetData>
     <row r="6" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="3:3" ht="15.75" x14ac:dyDescent="0.45">
+      <c r="C7" s="14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C8" s="15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="3:3" ht="15.75" x14ac:dyDescent="0.45">
-      <c r="C7" s="16" t="s">
+    <row r="9" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C9" s="16" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C10" s="15" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C8" s="17" t="s">
+    <row r="11" spans="3:3" ht="262.5" x14ac:dyDescent="0.45">
+      <c r="C11" s="16" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C9" s="18" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="10" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C10" s="17" t="s">
+    <row r="12" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C12" s="15" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="3:3" ht="262.5" x14ac:dyDescent="0.45">
-      <c r="C11" s="18" t="s">
+    <row r="13" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C13" s="16" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C12" s="17" t="s">
+    <row r="14" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C14" s="15" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C13" s="18" t="s">
+    <row r="15" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C15" s="16">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="16" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C16" s="15" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C14" s="17" t="s">
+    <row r="17" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C17" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C18" s="15" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C15" s="18">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="16" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C16" s="17" t="s">
+    <row r="19" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C19" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C20" s="15" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C17" s="18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C18" s="17" t="s">
+    <row r="21" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C21" s="15" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C19" s="18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C20" s="17" t="s">
+    <row r="22" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C22" s="16" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C23" s="15" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C21" s="17" t="s">
+    <row r="24" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C24" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C25" s="15" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="22" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C22" s="18" t="s">
+    <row r="26" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C26" s="16" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="23" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C23" s="17" t="s">
+    <row r="27" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C27" s="15" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C24" s="18" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="25" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C25" s="17" t="s">
+    <row r="28" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C28" s="16" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="26" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C26" s="18" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="27" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C27" s="17" t="s">
+    <row r="29" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C29" s="15" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C28" s="18" t="s">
+    <row r="30" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C30" s="15" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="29" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C29" s="17" t="s">
+    <row r="31" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C31" s="15" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="30" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C30" s="17" t="s">
+    <row r="32" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C32" s="16" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="31" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C31" s="17" t="s">
+    <row r="33" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
+      <c r="C33" s="15" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="32" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C32" s="18" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="33" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C33" s="17" t="s">
-        <v>55</v>
-      </c>
-    </row>
     <row r="34" spans="3:3" ht="18.75" x14ac:dyDescent="0.45">
-      <c r="C34" s="18">
+      <c r="C34" s="16">
         <v>1777195813120</v>
       </c>
     </row>

</xml_diff>